<commit_message>
indicator performance to json
</commit_message>
<xml_diff>
--- a/indicator-performance-table.xlsx
+++ b/indicator-performance-table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -594,6 +594,9 @@
   </si>
   <si>
     <t xml:space="preserve">This means that fewer people aged 18+ would prefer a mixed religion neighbourhood than did in 2020.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-24</t>
   </si>
 </sst>
 </file>
@@ -654,8 +657,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J105" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:J105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J157" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:J157"/>
   <tableColumns count="10">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="domain"/>
@@ -4295,6 +4298,1662 @@
         <v>170</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B106" t="s">
+        <v>10</v>
+      </c>
+      <c r="C106" t="s">
+        <v>11</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E106" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I106" t="s">
+        <v>15</v>
+      </c>
+      <c r="J106" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B107" t="s">
+        <v>10</v>
+      </c>
+      <c r="C107" t="s">
+        <v>17</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H107" s="3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I107" t="s">
+        <v>21</v>
+      </c>
+      <c r="J107" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B108" t="s">
+        <v>10</v>
+      </c>
+      <c r="C108" t="s">
+        <v>23</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="I108" t="s">
+        <v>21</v>
+      </c>
+      <c r="J108" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B109" t="s">
+        <v>10</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H109" s="3" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I109" t="s">
+        <v>30</v>
+      </c>
+      <c r="J109" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B110" t="s">
+        <v>32</v>
+      </c>
+      <c r="C110" t="s">
+        <v>33</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="I110" t="s">
+        <v>15</v>
+      </c>
+      <c r="J110" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B111" t="s">
+        <v>32</v>
+      </c>
+      <c r="C111" t="s">
+        <v>37</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E111" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I111" t="s">
+        <v>30</v>
+      </c>
+      <c r="J111" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B112" t="s">
+        <v>32</v>
+      </c>
+      <c r="C112" t="s">
+        <v>39</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="I112" t="s">
+        <v>21</v>
+      </c>
+      <c r="J112" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B113" t="s">
+        <v>32</v>
+      </c>
+      <c r="C113" t="s">
+        <v>44</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H113" s="3" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="I113" t="s">
+        <v>15</v>
+      </c>
+      <c r="J113" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B114" t="s">
+        <v>32</v>
+      </c>
+      <c r="C114" t="s">
+        <v>47</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E114" s="3" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="I114" t="s">
+        <v>30</v>
+      </c>
+      <c r="J114" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B115" t="s">
+        <v>32</v>
+      </c>
+      <c r="C115" t="s">
+        <v>50</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H115" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="I115" t="s">
+        <v>30</v>
+      </c>
+      <c r="J115" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B116" t="s">
+        <v>32</v>
+      </c>
+      <c r="C116" t="s">
+        <v>53</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E116" s="3" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="I116" t="s">
+        <v>21</v>
+      </c>
+      <c r="J116" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B117" t="s">
+        <v>32</v>
+      </c>
+      <c r="C117" t="s">
+        <v>56</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E117" s="3" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G117" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H117" s="3" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I117" t="s">
+        <v>30</v>
+      </c>
+      <c r="J117" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B118" t="s">
+        <v>32</v>
+      </c>
+      <c r="C118" t="s">
+        <v>59</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E118" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="I118" t="s">
+        <v>30</v>
+      </c>
+      <c r="J118" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B119" t="s">
+        <v>63</v>
+      </c>
+      <c r="C119" t="s">
+        <v>64</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E119" s="3" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G119" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H119" s="3" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="I119" t="s">
+        <v>15</v>
+      </c>
+      <c r="J119" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B120" t="s">
+        <v>63</v>
+      </c>
+      <c r="C120" t="s">
+        <v>67</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E120" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I120" t="s">
+        <v>30</v>
+      </c>
+      <c r="J120" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B121" t="s">
+        <v>63</v>
+      </c>
+      <c r="C121" t="s">
+        <v>71</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E121" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G121" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H121" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I121" t="s">
+        <v>30</v>
+      </c>
+      <c r="J121" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B122" t="s">
+        <v>63</v>
+      </c>
+      <c r="C122" t="s">
+        <v>73</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E122" s="3" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H122" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I122" t="s">
+        <v>21</v>
+      </c>
+      <c r="J122" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B123" t="s">
+        <v>75</v>
+      </c>
+      <c r="C123" t="s">
+        <v>76</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E123" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G123" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H123" s="3" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="I123" t="s">
+        <v>30</v>
+      </c>
+      <c r="J123" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B124" t="s">
+        <v>75</v>
+      </c>
+      <c r="C124" t="s">
+        <v>78</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E124" s="3" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="I124" t="s">
+        <v>21</v>
+      </c>
+      <c r="J124" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B125" t="s">
+        <v>75</v>
+      </c>
+      <c r="C125" t="s">
+        <v>83</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E125" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G125" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H125" s="3" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="I125" t="s">
+        <v>30</v>
+      </c>
+      <c r="J125" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B126" t="s">
+        <v>75</v>
+      </c>
+      <c r="C126" t="s">
+        <v>86</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E126" s="3" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G126" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H126" s="3" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="I126" t="s">
+        <v>15</v>
+      </c>
+      <c r="J126" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B127" t="s">
+        <v>75</v>
+      </c>
+      <c r="C127" t="s">
+        <v>89</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E127" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G127" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H127" s="3" t="n">
+        <v>181</v>
+      </c>
+      <c r="I127" t="s">
+        <v>21</v>
+      </c>
+      <c r="J127" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B128" t="s">
+        <v>75</v>
+      </c>
+      <c r="C128" t="s">
+        <v>94</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E128" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G128" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H128" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="I128" t="s">
+        <v>30</v>
+      </c>
+      <c r="J128" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B129" t="s">
+        <v>98</v>
+      </c>
+      <c r="C129" t="s">
+        <v>99</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E129" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H129" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="I129" t="s">
+        <v>15</v>
+      </c>
+      <c r="J129" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B130" t="s">
+        <v>98</v>
+      </c>
+      <c r="C130" t="s">
+        <v>101</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E130" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H130" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I130" t="s">
+        <v>30</v>
+      </c>
+      <c r="J130" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B131" t="s">
+        <v>98</v>
+      </c>
+      <c r="C131" t="s">
+        <v>104</v>
+      </c>
+      <c r="D131" s="3"/>
+      <c r="E131" s="3"/>
+      <c r="F131" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G131" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H131" s="3" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I131" t="s">
+        <v>61</v>
+      </c>
+      <c r="J131" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B132" t="s">
+        <v>98</v>
+      </c>
+      <c r="C132" t="s">
+        <v>106</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E132" s="3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I132" t="s">
+        <v>21</v>
+      </c>
+      <c r="J132" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B133" t="s">
+        <v>108</v>
+      </c>
+      <c r="C133" t="s">
+        <v>109</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E133" s="3" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G133" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H133" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I133" t="s">
+        <v>15</v>
+      </c>
+      <c r="J133" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B134" t="s">
+        <v>108</v>
+      </c>
+      <c r="C134" t="s">
+        <v>111</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E134" s="3" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H134" s="3" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="I134" t="s">
+        <v>15</v>
+      </c>
+      <c r="J134" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B135" t="s">
+        <v>108</v>
+      </c>
+      <c r="C135" t="s">
+        <v>114</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E135" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="G135" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H135" s="3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I135" t="s">
+        <v>15</v>
+      </c>
+      <c r="J135" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B136" t="s">
+        <v>108</v>
+      </c>
+      <c r="C136" t="s">
+        <v>117</v>
+      </c>
+      <c r="D136" s="3"/>
+      <c r="E136" s="3"/>
+      <c r="F136" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H136" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="I136" t="s">
+        <v>61</v>
+      </c>
+      <c r="J136" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B137" t="s">
+        <v>108</v>
+      </c>
+      <c r="C137" t="s">
+        <v>119</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E137" s="3" t="n">
+        <v>61.27</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G137" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H137" s="3" t="n">
+        <v>62.21</v>
+      </c>
+      <c r="I137" t="s">
+        <v>30</v>
+      </c>
+      <c r="J137" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B138" t="s">
+        <v>108</v>
+      </c>
+      <c r="C138" t="s">
+        <v>121</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="I138" t="s">
+        <v>15</v>
+      </c>
+      <c r="J138" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B139" t="s">
+        <v>108</v>
+      </c>
+      <c r="C139" t="s">
+        <v>123</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E139" s="3" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G139" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H139" s="3" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="I139" t="s">
+        <v>15</v>
+      </c>
+      <c r="J139" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B140" t="s">
+        <v>108</v>
+      </c>
+      <c r="C140" t="s">
+        <v>126</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E140" s="3" t="n">
+        <v>1170.4</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>1000.7</v>
+      </c>
+      <c r="I140" t="s">
+        <v>21</v>
+      </c>
+      <c r="J140" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B141" t="s">
+        <v>108</v>
+      </c>
+      <c r="C141" t="s">
+        <v>128</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E141" s="3" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G141" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H141" s="3" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="I141" t="s">
+        <v>15</v>
+      </c>
+      <c r="J141" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B142" t="s">
+        <v>131</v>
+      </c>
+      <c r="C142" t="s">
+        <v>132</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I142" t="s">
+        <v>30</v>
+      </c>
+      <c r="J142" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B143" t="s">
+        <v>131</v>
+      </c>
+      <c r="C143" t="s">
+        <v>134</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E143" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G143" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H143" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I143" t="s">
+        <v>30</v>
+      </c>
+      <c r="J143" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B144" t="s">
+        <v>131</v>
+      </c>
+      <c r="C144" t="s">
+        <v>136</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="I144" t="s">
+        <v>30</v>
+      </c>
+      <c r="J144" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B145" t="s">
+        <v>131</v>
+      </c>
+      <c r="C145" t="s">
+        <v>140</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E145" s="3" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G145" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H145" s="3" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="I145" t="s">
+        <v>21</v>
+      </c>
+      <c r="J145" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B146" t="s">
+        <v>131</v>
+      </c>
+      <c r="C146" t="s">
+        <v>142</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I146" t="s">
+        <v>30</v>
+      </c>
+      <c r="J146" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B147" t="s">
+        <v>145</v>
+      </c>
+      <c r="C147" t="s">
+        <v>146</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E147" s="3" t="n">
+        <v>68.4</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G147" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H147" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="I147" t="s">
+        <v>30</v>
+      </c>
+      <c r="J147" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B148" t="s">
+        <v>145</v>
+      </c>
+      <c r="C148" t="s">
+        <v>148</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I148" t="s">
+        <v>15</v>
+      </c>
+      <c r="J148" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B149" t="s">
+        <v>145</v>
+      </c>
+      <c r="C149" t="s">
+        <v>150</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G149" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H149" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I149" t="s">
+        <v>30</v>
+      </c>
+      <c r="J149" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B150" t="s">
+        <v>152</v>
+      </c>
+      <c r="C150" t="s">
+        <v>153</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G150" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="I150" t="s">
+        <v>30</v>
+      </c>
+      <c r="J150" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B151" t="s">
+        <v>152</v>
+      </c>
+      <c r="C151" t="s">
+        <v>154</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>10135</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G151" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H151" s="3" t="n">
+        <v>10855</v>
+      </c>
+      <c r="I151" t="s">
+        <v>21</v>
+      </c>
+      <c r="J151" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B152" t="s">
+        <v>152</v>
+      </c>
+      <c r="C152" t="s">
+        <v>156</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G152" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I152" t="s">
+        <v>30</v>
+      </c>
+      <c r="J152" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B153" t="s">
+        <v>152</v>
+      </c>
+      <c r="C153" t="s">
+        <v>159</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E153" s="3" t="n">
+        <v>30288</v>
+      </c>
+      <c r="F153" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G153" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H153" s="3" t="n">
+        <v>37635</v>
+      </c>
+      <c r="I153" t="s">
+        <v>21</v>
+      </c>
+      <c r="J153" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B154" t="s">
+        <v>161</v>
+      </c>
+      <c r="C154" t="s">
+        <v>162</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G154" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="I154" t="s">
+        <v>15</v>
+      </c>
+      <c r="J154" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B155" t="s">
+        <v>161</v>
+      </c>
+      <c r="C155" t="s">
+        <v>164</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E155" s="3" t="n">
+        <v>78.6</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G155" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H155" s="3" t="n">
+        <v>76.1</v>
+      </c>
+      <c r="I155" t="s">
+        <v>21</v>
+      </c>
+      <c r="J155" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B156" t="s">
+        <v>161</v>
+      </c>
+      <c r="C156" t="s">
+        <v>165</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G156" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="I156" t="s">
+        <v>30</v>
+      </c>
+      <c r="J156" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B157" t="s">
+        <v>161</v>
+      </c>
+      <c r="C157" t="s">
+        <v>168</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E157" s="3" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G157" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H157" s="3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I157" t="s">
+        <v>30</v>
+      </c>
+      <c r="J157" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
> to >= indicator performance
</commit_message>
<xml_diff>
--- a/indicator-performance-table.xlsx
+++ b/indicator-performance-table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -594,6 +594,9 @@
   </si>
   <si>
     <t xml:space="preserve">This means that fewer people aged 18+ would prefer a mixed religion neighbourhood than did in 2020.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The indicator shows that the percentage of households with accessible natural space within 400 metres has decreased since the comparision year 2023. 47.8 per cent of households are within 400m of greenspace &gt;2ha, and off-road trails in 2025.</t>
   </si>
   <si>
     <t xml:space="preserve">2020-24</t>
@@ -4580,10 +4583,10 @@
         <v>47.8</v>
       </c>
       <c r="I114" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="J114" t="s">
-        <v>49</v>
+        <v>194</v>
       </c>
     </row>
     <row r="115">
@@ -4990,7 +4993,7 @@
         <v>91</v>
       </c>
       <c r="G127" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H127" s="3" t="n">
         <v>181</v>
@@ -5028,10 +5031,10 @@
         <v>73</v>
       </c>
       <c r="I128" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="J128" t="s">
-        <v>97</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129">

</xml_diff>

<commit_message>
add last updated date
</commit_message>
<xml_diff>
--- a/indicator-performance-table.xlsx
+++ b/indicator-performance-table.xlsx
@@ -606,8 +606,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="2">
@@ -646,7 +645,7 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>

</xml_diff>

<commit_message>
change js links to github
</commit_message>
<xml_diff>
--- a/indicator-performance-table.xlsx
+++ b/indicator-performance-table.xlsx
@@ -659,8 +659,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J157" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:J157"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J209" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:J209"/>
   <tableColumns count="10">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="domain"/>
@@ -5956,6 +5956,1662 @@
         <v>170</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B158" t="s">
+        <v>10</v>
+      </c>
+      <c r="C158" t="s">
+        <v>11</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G158" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I158" t="s">
+        <v>15</v>
+      </c>
+      <c r="J158" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B159" t="s">
+        <v>10</v>
+      </c>
+      <c r="C159" t="s">
+        <v>17</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E159" s="3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F159" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G159" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H159" s="3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I159" t="s">
+        <v>21</v>
+      </c>
+      <c r="J159" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B160" t="s">
+        <v>10</v>
+      </c>
+      <c r="C160" t="s">
+        <v>23</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G160" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H160" s="3" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="I160" t="s">
+        <v>21</v>
+      </c>
+      <c r="J160" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B161" t="s">
+        <v>10</v>
+      </c>
+      <c r="C161" t="s">
+        <v>26</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E161" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F161" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G161" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H161" s="3" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I161" t="s">
+        <v>30</v>
+      </c>
+      <c r="J161" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B162" t="s">
+        <v>32</v>
+      </c>
+      <c r="C162" t="s">
+        <v>33</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G162" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="I162" t="s">
+        <v>15</v>
+      </c>
+      <c r="J162" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B163" t="s">
+        <v>32</v>
+      </c>
+      <c r="C163" t="s">
+        <v>37</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E163" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G163" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H163" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I163" t="s">
+        <v>30</v>
+      </c>
+      <c r="J163" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B164" t="s">
+        <v>32</v>
+      </c>
+      <c r="C164" t="s">
+        <v>39</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E164" s="3" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G164" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H164" s="3" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="I164" t="s">
+        <v>21</v>
+      </c>
+      <c r="J164" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B165" t="s">
+        <v>32</v>
+      </c>
+      <c r="C165" t="s">
+        <v>44</v>
+      </c>
+      <c r="D165" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E165" s="3" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="F165" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G165" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H165" s="3" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="I165" t="s">
+        <v>15</v>
+      </c>
+      <c r="J165" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B166" t="s">
+        <v>32</v>
+      </c>
+      <c r="C166" t="s">
+        <v>47</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E166" s="3" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G166" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H166" s="3" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="I166" t="s">
+        <v>21</v>
+      </c>
+      <c r="J166" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B167" t="s">
+        <v>32</v>
+      </c>
+      <c r="C167" t="s">
+        <v>50</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E167" s="3" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G167" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H167" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="I167" t="s">
+        <v>30</v>
+      </c>
+      <c r="J167" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B168" t="s">
+        <v>32</v>
+      </c>
+      <c r="C168" t="s">
+        <v>53</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E168" s="3" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G168" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H168" s="3" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="I168" t="s">
+        <v>21</v>
+      </c>
+      <c r="J168" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B169" t="s">
+        <v>32</v>
+      </c>
+      <c r="C169" t="s">
+        <v>56</v>
+      </c>
+      <c r="D169" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E169" s="3" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G169" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H169" s="3" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I169" t="s">
+        <v>30</v>
+      </c>
+      <c r="J169" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B170" t="s">
+        <v>32</v>
+      </c>
+      <c r="C170" t="s">
+        <v>59</v>
+      </c>
+      <c r="D170" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E170" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G170" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H170" s="3" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="I170" t="s">
+        <v>30</v>
+      </c>
+      <c r="J170" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B171" t="s">
+        <v>63</v>
+      </c>
+      <c r="C171" t="s">
+        <v>64</v>
+      </c>
+      <c r="D171" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E171" s="3" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="F171" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G171" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H171" s="3" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="I171" t="s">
+        <v>15</v>
+      </c>
+      <c r="J171" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B172" t="s">
+        <v>63</v>
+      </c>
+      <c r="C172" t="s">
+        <v>67</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E172" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G172" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H172" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I172" t="s">
+        <v>30</v>
+      </c>
+      <c r="J172" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B173" t="s">
+        <v>63</v>
+      </c>
+      <c r="C173" t="s">
+        <v>71</v>
+      </c>
+      <c r="D173" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E173" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F173" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G173" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H173" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I173" t="s">
+        <v>30</v>
+      </c>
+      <c r="J173" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B174" t="s">
+        <v>63</v>
+      </c>
+      <c r="C174" t="s">
+        <v>73</v>
+      </c>
+      <c r="D174" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E174" s="3" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="F174" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G174" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H174" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I174" t="s">
+        <v>21</v>
+      </c>
+      <c r="J174" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B175" t="s">
+        <v>75</v>
+      </c>
+      <c r="C175" t="s">
+        <v>76</v>
+      </c>
+      <c r="D175" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E175" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="F175" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G175" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H175" s="3" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="I175" t="s">
+        <v>30</v>
+      </c>
+      <c r="J175" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B176" t="s">
+        <v>75</v>
+      </c>
+      <c r="C176" t="s">
+        <v>78</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E176" s="3" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="F176" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G176" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H176" s="3" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="I176" t="s">
+        <v>21</v>
+      </c>
+      <c r="J176" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B177" t="s">
+        <v>75</v>
+      </c>
+      <c r="C177" t="s">
+        <v>83</v>
+      </c>
+      <c r="D177" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E177" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F177" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G177" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H177" s="3" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="I177" t="s">
+        <v>30</v>
+      </c>
+      <c r="J177" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B178" t="s">
+        <v>75</v>
+      </c>
+      <c r="C178" t="s">
+        <v>86</v>
+      </c>
+      <c r="D178" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E178" s="3" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F178" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G178" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H178" s="3" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="I178" t="s">
+        <v>15</v>
+      </c>
+      <c r="J178" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B179" t="s">
+        <v>75</v>
+      </c>
+      <c r="C179" t="s">
+        <v>89</v>
+      </c>
+      <c r="D179" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E179" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="F179" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G179" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="H179" s="3" t="n">
+        <v>181</v>
+      </c>
+      <c r="I179" t="s">
+        <v>21</v>
+      </c>
+      <c r="J179" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B180" t="s">
+        <v>75</v>
+      </c>
+      <c r="C180" t="s">
+        <v>94</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E180" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G180" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H180" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="I180" t="s">
+        <v>21</v>
+      </c>
+      <c r="J180" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B181" t="s">
+        <v>98</v>
+      </c>
+      <c r="C181" t="s">
+        <v>99</v>
+      </c>
+      <c r="D181" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E181" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F181" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G181" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H181" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="I181" t="s">
+        <v>15</v>
+      </c>
+      <c r="J181" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B182" t="s">
+        <v>98</v>
+      </c>
+      <c r="C182" t="s">
+        <v>101</v>
+      </c>
+      <c r="D182" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E182" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F182" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G182" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H182" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I182" t="s">
+        <v>30</v>
+      </c>
+      <c r="J182" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B183" t="s">
+        <v>98</v>
+      </c>
+      <c r="C183" t="s">
+        <v>104</v>
+      </c>
+      <c r="D183" s="3"/>
+      <c r="E183" s="3"/>
+      <c r="F183" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G183" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H183" s="3" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I183" t="s">
+        <v>61</v>
+      </c>
+      <c r="J183" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B184" t="s">
+        <v>98</v>
+      </c>
+      <c r="C184" t="s">
+        <v>106</v>
+      </c>
+      <c r="D184" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E184" s="3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F184" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G184" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H184" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I184" t="s">
+        <v>21</v>
+      </c>
+      <c r="J184" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B185" t="s">
+        <v>108</v>
+      </c>
+      <c r="C185" t="s">
+        <v>109</v>
+      </c>
+      <c r="D185" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E185" s="3" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="F185" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G185" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H185" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I185" t="s">
+        <v>15</v>
+      </c>
+      <c r="J185" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B186" t="s">
+        <v>108</v>
+      </c>
+      <c r="C186" t="s">
+        <v>111</v>
+      </c>
+      <c r="D186" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E186" s="3" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="F186" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G186" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H186" s="3" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="I186" t="s">
+        <v>15</v>
+      </c>
+      <c r="J186" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B187" t="s">
+        <v>108</v>
+      </c>
+      <c r="C187" t="s">
+        <v>114</v>
+      </c>
+      <c r="D187" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E187" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F187" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="G187" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H187" s="3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I187" t="s">
+        <v>15</v>
+      </c>
+      <c r="J187" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B188" t="s">
+        <v>108</v>
+      </c>
+      <c r="C188" t="s">
+        <v>117</v>
+      </c>
+      <c r="D188" s="3"/>
+      <c r="E188" s="3"/>
+      <c r="F188" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G188" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H188" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="I188" t="s">
+        <v>61</v>
+      </c>
+      <c r="J188" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B189" t="s">
+        <v>108</v>
+      </c>
+      <c r="C189" t="s">
+        <v>119</v>
+      </c>
+      <c r="D189" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E189" s="3" t="n">
+        <v>61.27</v>
+      </c>
+      <c r="F189" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G189" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H189" s="3" t="n">
+        <v>62.21</v>
+      </c>
+      <c r="I189" t="s">
+        <v>30</v>
+      </c>
+      <c r="J189" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B190" t="s">
+        <v>108</v>
+      </c>
+      <c r="C190" t="s">
+        <v>121</v>
+      </c>
+      <c r="D190" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E190" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="F190" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G190" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H190" s="3" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="I190" t="s">
+        <v>15</v>
+      </c>
+      <c r="J190" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B191" t="s">
+        <v>108</v>
+      </c>
+      <c r="C191" t="s">
+        <v>123</v>
+      </c>
+      <c r="D191" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E191" s="3" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="F191" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G191" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H191" s="3" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="I191" t="s">
+        <v>15</v>
+      </c>
+      <c r="J191" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B192" t="s">
+        <v>108</v>
+      </c>
+      <c r="C192" t="s">
+        <v>126</v>
+      </c>
+      <c r="D192" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E192" s="3" t="n">
+        <v>1170.4</v>
+      </c>
+      <c r="F192" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G192" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H192" s="3" t="n">
+        <v>1000.7</v>
+      </c>
+      <c r="I192" t="s">
+        <v>21</v>
+      </c>
+      <c r="J192" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B193" t="s">
+        <v>108</v>
+      </c>
+      <c r="C193" t="s">
+        <v>128</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E193" s="3" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="F193" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G193" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H193" s="3" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="I193" t="s">
+        <v>15</v>
+      </c>
+      <c r="J193" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B194" t="s">
+        <v>131</v>
+      </c>
+      <c r="C194" t="s">
+        <v>132</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E194" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G194" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H194" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I194" t="s">
+        <v>30</v>
+      </c>
+      <c r="J194" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B195" t="s">
+        <v>131</v>
+      </c>
+      <c r="C195" t="s">
+        <v>134</v>
+      </c>
+      <c r="D195" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E195" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="F195" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G195" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H195" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I195" t="s">
+        <v>30</v>
+      </c>
+      <c r="J195" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B196" t="s">
+        <v>131</v>
+      </c>
+      <c r="C196" t="s">
+        <v>136</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E196" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="F196" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G196" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H196" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="I196" t="s">
+        <v>30</v>
+      </c>
+      <c r="J196" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B197" t="s">
+        <v>131</v>
+      </c>
+      <c r="C197" t="s">
+        <v>140</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E197" s="3" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F197" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G197" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H197" s="3" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="I197" t="s">
+        <v>21</v>
+      </c>
+      <c r="J197" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B198" t="s">
+        <v>131</v>
+      </c>
+      <c r="C198" t="s">
+        <v>142</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E198" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F198" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G198" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H198" s="3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I198" t="s">
+        <v>30</v>
+      </c>
+      <c r="J198" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B199" t="s">
+        <v>145</v>
+      </c>
+      <c r="C199" t="s">
+        <v>146</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E199" s="3" t="n">
+        <v>68.4</v>
+      </c>
+      <c r="F199" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G199" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H199" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="I199" t="s">
+        <v>30</v>
+      </c>
+      <c r="J199" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B200" t="s">
+        <v>145</v>
+      </c>
+      <c r="C200" t="s">
+        <v>148</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E200" s="3" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="F200" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G200" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H200" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I200" t="s">
+        <v>15</v>
+      </c>
+      <c r="J200" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B201" t="s">
+        <v>145</v>
+      </c>
+      <c r="C201" t="s">
+        <v>150</v>
+      </c>
+      <c r="D201" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E201" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="F201" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G201" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H201" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I201" t="s">
+        <v>30</v>
+      </c>
+      <c r="J201" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B202" t="s">
+        <v>152</v>
+      </c>
+      <c r="C202" t="s">
+        <v>153</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E202" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F202" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G202" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H202" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="I202" t="s">
+        <v>30</v>
+      </c>
+      <c r="J202" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B203" t="s">
+        <v>152</v>
+      </c>
+      <c r="C203" t="s">
+        <v>154</v>
+      </c>
+      <c r="D203" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E203" s="3" t="n">
+        <v>10135</v>
+      </c>
+      <c r="F203" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G203" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H203" s="3" t="n">
+        <v>10855</v>
+      </c>
+      <c r="I203" t="s">
+        <v>21</v>
+      </c>
+      <c r="J203" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B204" t="s">
+        <v>152</v>
+      </c>
+      <c r="C204" t="s">
+        <v>156</v>
+      </c>
+      <c r="D204" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E204" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F204" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G204" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H204" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I204" t="s">
+        <v>30</v>
+      </c>
+      <c r="J204" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B205" t="s">
+        <v>152</v>
+      </c>
+      <c r="C205" t="s">
+        <v>159</v>
+      </c>
+      <c r="D205" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E205" s="3" t="n">
+        <v>30288</v>
+      </c>
+      <c r="F205" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G205" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H205" s="3" t="n">
+        <v>37635</v>
+      </c>
+      <c r="I205" t="s">
+        <v>21</v>
+      </c>
+      <c r="J205" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B206" t="s">
+        <v>161</v>
+      </c>
+      <c r="C206" t="s">
+        <v>162</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E206" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F206" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G206" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H206" s="3" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="I206" t="s">
+        <v>15</v>
+      </c>
+      <c r="J206" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B207" t="s">
+        <v>161</v>
+      </c>
+      <c r="C207" t="s">
+        <v>164</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E207" s="3" t="n">
+        <v>78.6</v>
+      </c>
+      <c r="F207" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G207" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H207" s="3" t="n">
+        <v>76.1</v>
+      </c>
+      <c r="I207" t="s">
+        <v>21</v>
+      </c>
+      <c r="J207" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B208" t="s">
+        <v>161</v>
+      </c>
+      <c r="C208" t="s">
+        <v>165</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E208" s="3" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F208" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G208" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H208" s="3" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="I208" t="s">
+        <v>30</v>
+      </c>
+      <c r="J208" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B209" t="s">
+        <v>161</v>
+      </c>
+      <c r="C209" t="s">
+        <v>168</v>
+      </c>
+      <c r="D209" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E209" s="3" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F209" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G209" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H209" s="3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I209" t="s">
+        <v>30</v>
+      </c>
+      <c r="J209" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
run back up data portal script
</commit_message>
<xml_diff>
--- a/indicator-performance-table.xlsx
+++ b/indicator-performance-table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="198">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -600,6 +600,12 @@
   </si>
   <si>
     <t xml:space="preserve">2020-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025/26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026</t>
   </si>
 </sst>
 </file>
@@ -659,8 +665,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J209" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:J209"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J261" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:J261"/>
   <tableColumns count="10">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="domain"/>
@@ -7612,6 +7618,1662 @@
         <v>170</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B210" t="s">
+        <v>10</v>
+      </c>
+      <c r="C210" t="s">
+        <v>11</v>
+      </c>
+      <c r="D210" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E210" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="F210" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G210" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H210" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I210" t="s">
+        <v>15</v>
+      </c>
+      <c r="J210" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B211" t="s">
+        <v>10</v>
+      </c>
+      <c r="C211" t="s">
+        <v>17</v>
+      </c>
+      <c r="D211" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E211" s="3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F211" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G211" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H211" s="3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I211" t="s">
+        <v>21</v>
+      </c>
+      <c r="J211" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B212" t="s">
+        <v>10</v>
+      </c>
+      <c r="C212" t="s">
+        <v>23</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E212" s="3" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G212" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H212" s="3" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="I212" t="s">
+        <v>21</v>
+      </c>
+      <c r="J212" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B213" t="s">
+        <v>10</v>
+      </c>
+      <c r="C213" t="s">
+        <v>26</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E213" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G213" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H213" s="3" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I213" t="s">
+        <v>30</v>
+      </c>
+      <c r="J213" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B214" t="s">
+        <v>32</v>
+      </c>
+      <c r="C214" t="s">
+        <v>33</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E214" s="3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F214" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G214" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H214" s="3" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="I214" t="s">
+        <v>15</v>
+      </c>
+      <c r="J214" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B215" t="s">
+        <v>32</v>
+      </c>
+      <c r="C215" t="s">
+        <v>37</v>
+      </c>
+      <c r="D215" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E215" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F215" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G215" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H215" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I215" t="s">
+        <v>21</v>
+      </c>
+      <c r="J215" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B216" t="s">
+        <v>32</v>
+      </c>
+      <c r="C216" t="s">
+        <v>39</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E216" s="3" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="F216" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G216" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H216" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="I216" t="s">
+        <v>21</v>
+      </c>
+      <c r="J216" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B217" t="s">
+        <v>32</v>
+      </c>
+      <c r="C217" t="s">
+        <v>44</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E217" s="3" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="F217" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G217" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H217" s="3" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="I217" t="s">
+        <v>15</v>
+      </c>
+      <c r="J217" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B218" t="s">
+        <v>32</v>
+      </c>
+      <c r="C218" t="s">
+        <v>47</v>
+      </c>
+      <c r="D218" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E218" s="3" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G218" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="H218" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="I218" t="s">
+        <v>21</v>
+      </c>
+      <c r="J218" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B219" t="s">
+        <v>32</v>
+      </c>
+      <c r="C219" t="s">
+        <v>50</v>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E219" s="3" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F219" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G219" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H219" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="I219" t="s">
+        <v>30</v>
+      </c>
+      <c r="J219" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B220" t="s">
+        <v>32</v>
+      </c>
+      <c r="C220" t="s">
+        <v>53</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E220" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G220" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H220" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="I220" t="s">
+        <v>21</v>
+      </c>
+      <c r="J220" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B221" t="s">
+        <v>32</v>
+      </c>
+      <c r="C221" t="s">
+        <v>56</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E221" s="3" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G221" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H221" s="3" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="I221" t="s">
+        <v>30</v>
+      </c>
+      <c r="J221" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B222" t="s">
+        <v>32</v>
+      </c>
+      <c r="C222" t="s">
+        <v>59</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E222" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G222" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H222" s="3" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="I222" t="s">
+        <v>30</v>
+      </c>
+      <c r="J222" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B223" t="s">
+        <v>63</v>
+      </c>
+      <c r="C223" t="s">
+        <v>64</v>
+      </c>
+      <c r="D223" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E223" s="3" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G223" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H223" s="3" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="I223" t="s">
+        <v>15</v>
+      </c>
+      <c r="J223" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B224" t="s">
+        <v>63</v>
+      </c>
+      <c r="C224" t="s">
+        <v>67</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E224" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G224" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H224" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I224" t="s">
+        <v>30</v>
+      </c>
+      <c r="J224" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B225" t="s">
+        <v>63</v>
+      </c>
+      <c r="C225" t="s">
+        <v>71</v>
+      </c>
+      <c r="D225" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E225" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F225" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G225" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H225" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I225" t="s">
+        <v>30</v>
+      </c>
+      <c r="J225" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B226" t="s">
+        <v>63</v>
+      </c>
+      <c r="C226" t="s">
+        <v>73</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E226" s="3" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="F226" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G226" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H226" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I226" t="s">
+        <v>21</v>
+      </c>
+      <c r="J226" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B227" t="s">
+        <v>75</v>
+      </c>
+      <c r="C227" t="s">
+        <v>76</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E227" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="F227" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G227" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H227" s="3" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="I227" t="s">
+        <v>30</v>
+      </c>
+      <c r="J227" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B228" t="s">
+        <v>75</v>
+      </c>
+      <c r="C228" t="s">
+        <v>78</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E228" s="3" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="F228" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G228" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H228" s="3" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="I228" t="s">
+        <v>21</v>
+      </c>
+      <c r="J228" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B229" t="s">
+        <v>75</v>
+      </c>
+      <c r="C229" t="s">
+        <v>83</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E229" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F229" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G229" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H229" s="3" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="I229" t="s">
+        <v>30</v>
+      </c>
+      <c r="J229" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B230" t="s">
+        <v>75</v>
+      </c>
+      <c r="C230" t="s">
+        <v>86</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E230" s="3" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F230" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G230" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H230" s="3" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="I230" t="s">
+        <v>15</v>
+      </c>
+      <c r="J230" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B231" t="s">
+        <v>75</v>
+      </c>
+      <c r="C231" t="s">
+        <v>89</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E231" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="F231" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G231" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="H231" s="3" t="n">
+        <v>181</v>
+      </c>
+      <c r="I231" t="s">
+        <v>21</v>
+      </c>
+      <c r="J231" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B232" t="s">
+        <v>75</v>
+      </c>
+      <c r="C232" t="s">
+        <v>94</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E232" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="F232" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G232" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H232" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="I232" t="s">
+        <v>21</v>
+      </c>
+      <c r="J232" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B233" t="s">
+        <v>98</v>
+      </c>
+      <c r="C233" t="s">
+        <v>99</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E233" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F233" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G233" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H233" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="I233" t="s">
+        <v>15</v>
+      </c>
+      <c r="J233" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B234" t="s">
+        <v>98</v>
+      </c>
+      <c r="C234" t="s">
+        <v>101</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E234" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F234" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G234" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H234" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I234" t="s">
+        <v>30</v>
+      </c>
+      <c r="J234" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B235" t="s">
+        <v>98</v>
+      </c>
+      <c r="C235" t="s">
+        <v>104</v>
+      </c>
+      <c r="D235" s="3"/>
+      <c r="E235" s="3"/>
+      <c r="F235" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G235" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H235" s="3" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I235" t="s">
+        <v>61</v>
+      </c>
+      <c r="J235" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B236" t="s">
+        <v>98</v>
+      </c>
+      <c r="C236" t="s">
+        <v>106</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E236" s="3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F236" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G236" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H236" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I236" t="s">
+        <v>21</v>
+      </c>
+      <c r="J236" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B237" t="s">
+        <v>108</v>
+      </c>
+      <c r="C237" t="s">
+        <v>109</v>
+      </c>
+      <c r="D237" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E237" s="3" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="F237" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G237" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H237" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I237" t="s">
+        <v>15</v>
+      </c>
+      <c r="J237" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B238" t="s">
+        <v>108</v>
+      </c>
+      <c r="C238" t="s">
+        <v>111</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E238" s="3" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="F238" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G238" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H238" s="3" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="I238" t="s">
+        <v>15</v>
+      </c>
+      <c r="J238" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B239" t="s">
+        <v>108</v>
+      </c>
+      <c r="C239" t="s">
+        <v>114</v>
+      </c>
+      <c r="D239" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E239" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F239" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="G239" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H239" s="3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I239" t="s">
+        <v>15</v>
+      </c>
+      <c r="J239" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B240" t="s">
+        <v>108</v>
+      </c>
+      <c r="C240" t="s">
+        <v>117</v>
+      </c>
+      <c r="D240" s="3"/>
+      <c r="E240" s="3"/>
+      <c r="F240" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G240" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H240" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="I240" t="s">
+        <v>61</v>
+      </c>
+      <c r="J240" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B241" t="s">
+        <v>108</v>
+      </c>
+      <c r="C241" t="s">
+        <v>119</v>
+      </c>
+      <c r="D241" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E241" s="3" t="n">
+        <v>61.27</v>
+      </c>
+      <c r="F241" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G241" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H241" s="3" t="n">
+        <v>62.21</v>
+      </c>
+      <c r="I241" t="s">
+        <v>30</v>
+      </c>
+      <c r="J241" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B242" t="s">
+        <v>108</v>
+      </c>
+      <c r="C242" t="s">
+        <v>121</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E242" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="F242" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G242" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H242" s="3" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="I242" t="s">
+        <v>15</v>
+      </c>
+      <c r="J242" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B243" t="s">
+        <v>108</v>
+      </c>
+      <c r="C243" t="s">
+        <v>123</v>
+      </c>
+      <c r="D243" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E243" s="3" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="F243" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G243" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H243" s="3" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="I243" t="s">
+        <v>15</v>
+      </c>
+      <c r="J243" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B244" t="s">
+        <v>108</v>
+      </c>
+      <c r="C244" t="s">
+        <v>126</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E244" s="3" t="n">
+        <v>1170.4</v>
+      </c>
+      <c r="F244" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G244" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H244" s="3" t="n">
+        <v>1000.7</v>
+      </c>
+      <c r="I244" t="s">
+        <v>21</v>
+      </c>
+      <c r="J244" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B245" t="s">
+        <v>108</v>
+      </c>
+      <c r="C245" t="s">
+        <v>128</v>
+      </c>
+      <c r="D245" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E245" s="3" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="F245" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G245" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H245" s="3" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="I245" t="s">
+        <v>15</v>
+      </c>
+      <c r="J245" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B246" t="s">
+        <v>131</v>
+      </c>
+      <c r="C246" t="s">
+        <v>132</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E246" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G246" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H246" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I246" t="s">
+        <v>30</v>
+      </c>
+      <c r="J246" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B247" t="s">
+        <v>131</v>
+      </c>
+      <c r="C247" t="s">
+        <v>134</v>
+      </c>
+      <c r="D247" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E247" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="F247" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G247" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H247" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I247" t="s">
+        <v>30</v>
+      </c>
+      <c r="J247" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B248" t="s">
+        <v>131</v>
+      </c>
+      <c r="C248" t="s">
+        <v>136</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E248" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="F248" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G248" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H248" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="I248" t="s">
+        <v>30</v>
+      </c>
+      <c r="J248" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B249" t="s">
+        <v>131</v>
+      </c>
+      <c r="C249" t="s">
+        <v>140</v>
+      </c>
+      <c r="D249" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E249" s="3" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F249" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G249" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H249" s="3" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="I249" t="s">
+        <v>21</v>
+      </c>
+      <c r="J249" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B250" t="s">
+        <v>131</v>
+      </c>
+      <c r="C250" t="s">
+        <v>142</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E250" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F250" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G250" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H250" s="3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I250" t="s">
+        <v>30</v>
+      </c>
+      <c r="J250" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B251" t="s">
+        <v>145</v>
+      </c>
+      <c r="C251" t="s">
+        <v>146</v>
+      </c>
+      <c r="D251" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E251" s="3" t="n">
+        <v>68.4</v>
+      </c>
+      <c r="F251" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G251" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H251" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="I251" t="s">
+        <v>30</v>
+      </c>
+      <c r="J251" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B252" t="s">
+        <v>145</v>
+      </c>
+      <c r="C252" t="s">
+        <v>148</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E252" s="3" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="F252" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G252" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H252" s="3" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="I252" t="s">
+        <v>15</v>
+      </c>
+      <c r="J252" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B253" t="s">
+        <v>145</v>
+      </c>
+      <c r="C253" t="s">
+        <v>150</v>
+      </c>
+      <c r="D253" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E253" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="F253" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G253" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H253" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I253" t="s">
+        <v>30</v>
+      </c>
+      <c r="J253" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B254" t="s">
+        <v>152</v>
+      </c>
+      <c r="C254" t="s">
+        <v>153</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E254" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F254" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G254" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H254" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="I254" t="s">
+        <v>30</v>
+      </c>
+      <c r="J254" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B255" t="s">
+        <v>152</v>
+      </c>
+      <c r="C255" t="s">
+        <v>154</v>
+      </c>
+      <c r="D255" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E255" s="3" t="n">
+        <v>10135</v>
+      </c>
+      <c r="F255" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G255" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H255" s="3" t="n">
+        <v>10855</v>
+      </c>
+      <c r="I255" t="s">
+        <v>21</v>
+      </c>
+      <c r="J255" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B256" t="s">
+        <v>152</v>
+      </c>
+      <c r="C256" t="s">
+        <v>156</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E256" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F256" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G256" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H256" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I256" t="s">
+        <v>30</v>
+      </c>
+      <c r="J256" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B257" t="s">
+        <v>152</v>
+      </c>
+      <c r="C257" t="s">
+        <v>159</v>
+      </c>
+      <c r="D257" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E257" s="3" t="n">
+        <v>30288</v>
+      </c>
+      <c r="F257" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G257" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H257" s="3" t="n">
+        <v>37635</v>
+      </c>
+      <c r="I257" t="s">
+        <v>21</v>
+      </c>
+      <c r="J257" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B258" t="s">
+        <v>161</v>
+      </c>
+      <c r="C258" t="s">
+        <v>162</v>
+      </c>
+      <c r="D258" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E258" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F258" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G258" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H258" s="3" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="I258" t="s">
+        <v>15</v>
+      </c>
+      <c r="J258" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B259" t="s">
+        <v>161</v>
+      </c>
+      <c r="C259" t="s">
+        <v>164</v>
+      </c>
+      <c r="D259" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E259" s="3" t="n">
+        <v>78.6</v>
+      </c>
+      <c r="F259" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G259" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H259" s="3" t="n">
+        <v>76.1</v>
+      </c>
+      <c r="I259" t="s">
+        <v>21</v>
+      </c>
+      <c r="J259" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B260" t="s">
+        <v>161</v>
+      </c>
+      <c r="C260" t="s">
+        <v>165</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E260" s="3" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F260" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G260" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H260" s="3" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="I260" t="s">
+        <v>30</v>
+      </c>
+      <c r="J260" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B261" t="s">
+        <v>161</v>
+      </c>
+      <c r="C261" t="s">
+        <v>168</v>
+      </c>
+      <c r="D261" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E261" s="3" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F261" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G261" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H261" s="3" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="I261" t="s">
+        <v>30</v>
+      </c>
+      <c r="J261" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>